<commit_message>
Rebuild sample workbooks from live SEC filings
</commit_message>
<xml_diff>
--- a/samples/AAPL_company_profile.xlsx
+++ b/samples/AAPL_company_profile.xlsx
@@ -662,19 +662,19 @@
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>260174000000</v>
+        <v>365817000000</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>274515000000</v>
+        <v>394328000000</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>365817000000</v>
+        <v>383285000000</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>394328000000</v>
+        <v>391035000000</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>383285000000</v>
+        <v>416161000000</v>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
@@ -717,19 +717,19 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>98392000000</v>
+        <v>152836000000</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>104956000000</v>
+        <v>170782000000</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>152836000000</v>
+        <v>169148000000</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>170782000000</v>
+        <v>180683000000</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>169148000000</v>
+        <v>195201000000</v>
       </c>
       <c r="J10" s="11" t="inlineStr">
         <is>
@@ -771,19 +771,19 @@
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>63930000000</v>
+        <v>108949000000</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>66288000000</v>
+        <v>119437000000</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>108949000000</v>
+        <v>114301000000</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>119437000000</v>
+        <v>123216000000</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>114301000000</v>
+        <v>133050000000</v>
       </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
@@ -825,19 +825,19 @@
         </is>
       </c>
       <c r="D14" s="10" t="n">
-        <v>55256000000</v>
+        <v>94680000000</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>57411000000</v>
+        <v>99803000000</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>94680000000</v>
+        <v>96995000000</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>99803000000</v>
+        <v>93736000000</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>96995000000</v>
+        <v>112010000000</v>
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
@@ -891,19 +891,19 @@
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>2.97</v>
+        <v>5.61</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>3.28</v>
+        <v>6.11</v>
       </c>
       <c r="F18" s="15" t="n">
-        <v>5.61</v>
+        <v>6.13</v>
       </c>
       <c r="G18" s="15" t="n">
-        <v>6.11</v>
+        <v>6.08</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>6.13</v>
+        <v>7.46</v>
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
@@ -918,19 +918,19 @@
         </is>
       </c>
       <c r="D19" s="16" t="n">
-        <v>18595651000</v>
+        <v>16864919000</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>17528214000</v>
+        <v>16325819000</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>16864919000</v>
+        <v>15812547000</v>
       </c>
       <c r="G19" s="16" t="n">
-        <v>16325819000</v>
+        <v>15408095000</v>
       </c>
       <c r="H19" s="16" t="n">
-        <v>15812547000</v>
+        <v>15004697000</v>
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
@@ -957,19 +957,19 @@
         </is>
       </c>
       <c r="D22" s="10" t="n">
-        <v>69391000000</v>
+        <v>104038000000</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>80674000000</v>
+        <v>122151000000</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>104038000000</v>
+        <v>110543000000</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>122151000000</v>
+        <v>118254000000</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>110543000000</v>
+        <v>111482000000</v>
       </c>
       <c r="J22" s="11" t="inlineStr">
         <is>
@@ -984,19 +984,19 @@
         </is>
       </c>
       <c r="D23" s="10" t="n">
-        <v>10495000000</v>
+        <v>11085000000</v>
       </c>
       <c r="E23" s="10" t="n">
-        <v>7309000000</v>
+        <v>10708000000</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>11085000000</v>
+        <v>10959000000</v>
       </c>
       <c r="G23" s="10" t="n">
-        <v>10708000000</v>
+        <v>9447000000</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>10959000000</v>
+        <v>12715000000</v>
       </c>
       <c r="J23" s="11" t="inlineStr">
         <is>
@@ -1077,19 +1077,19 @@
         </is>
       </c>
       <c r="D28" s="10" t="n">
-        <v>38016000000</v>
+        <v>34940000000</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>34940000000</v>
+        <v>23646000000</v>
       </c>
       <c r="F28" s="10" t="n">
-        <v>23646000000</v>
+        <v>29965000000</v>
       </c>
       <c r="G28" s="10" t="n">
-        <v>29965000000</v>
+        <v>29943000000</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>29943000000</v>
+        <v>35934000000</v>
       </c>
       <c r="J28" s="11" t="inlineStr">
         <is>
@@ -1136,19 +1136,19 @@
         </is>
       </c>
       <c r="D30" s="10" t="n">
-        <v>107440000000</v>
+        <v>118719000000</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>118719000000</v>
+        <v>110087000000</v>
       </c>
       <c r="F30" s="10" t="n">
-        <v>110087000000</v>
+        <v>105103000000</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>105103000000</v>
+        <v>96662000000</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>96662000000</v>
+        <v>90678000000</v>
       </c>
       <c r="J30" s="11" t="inlineStr">
         <is>
@@ -1163,19 +1163,19 @@
         </is>
       </c>
       <c r="D31" s="20" t="n">
-        <v>69424000000</v>
+        <v>83779000000</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>83779000000</v>
+        <v>86441000000</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>86441000000</v>
+        <v>75138000000</v>
       </c>
       <c r="G31" s="20" t="n">
-        <v>75138000000</v>
+        <v>66719000000</v>
       </c>
       <c r="H31" s="20" t="n">
-        <v>66719000000</v>
+        <v>54744000000</v>
       </c>
       <c r="J31" s="11" t="inlineStr">
         <is>
@@ -1190,19 +1190,19 @@
         </is>
       </c>
       <c r="D32" s="10" t="n">
-        <v>107147000000</v>
+        <v>63090000000</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>90488000000</v>
+        <v>50672000000</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>65339000000</v>
+        <v>62146000000</v>
       </c>
       <c r="G32" s="10" t="n">
-        <v>63090000000</v>
+        <v>56950000000</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>50672000000</v>
+        <v>73733000000</v>
       </c>
       <c r="J32" s="11" t="inlineStr">
         <is>
@@ -1330,19 +1330,19 @@
         </is>
       </c>
       <c r="D7" s="20" t="n">
-        <v>260174000000</v>
+        <v>365817000000</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>274515000000</v>
+        <v>394328000000</v>
       </c>
       <c r="F7" s="20" t="n">
-        <v>365817000000</v>
+        <v>383285000000</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>394328000000</v>
+        <v>391035000000</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>383285000000</v>
+        <v>416161000000</v>
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
@@ -1385,19 +1385,19 @@
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>161782000000</v>
+        <v>212981000000</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>169559000000</v>
+        <v>223546000000</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>212981000000</v>
+        <v>214137000000</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>223546000000</v>
+        <v>210352000000</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>214137000000</v>
+        <v>220960000000</v>
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
@@ -1412,19 +1412,19 @@
         </is>
       </c>
       <c r="D10" s="20" t="n">
-        <v>98392000000</v>
+        <v>152836000000</v>
       </c>
       <c r="E10" s="20" t="n">
-        <v>104956000000</v>
+        <v>170782000000</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>152836000000</v>
+        <v>169148000000</v>
       </c>
       <c r="G10" s="20" t="n">
-        <v>170782000000</v>
+        <v>180683000000</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>169148000000</v>
+        <v>195201000000</v>
       </c>
       <c r="J10" s="11" t="inlineStr">
         <is>
@@ -1466,19 +1466,19 @@
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>16217000000</v>
+        <v>21914000000</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>18752000000</v>
+        <v>26251000000</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>21914000000</v>
+        <v>29915000000</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>26251000000</v>
+        <v>31370000000</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>29915000000</v>
+        <v>34550000000</v>
       </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
@@ -1493,19 +1493,19 @@
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>18245000000</v>
+        <v>21973000000</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>19916000000</v>
+        <v>25094000000</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>21973000000</v>
+        <v>24932000000</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>25094000000</v>
+        <v>26097000000</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>24932000000</v>
+        <v>27601000000</v>
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
@@ -1520,19 +1520,19 @@
         </is>
       </c>
       <c r="D14" s="20" t="n">
-        <v>63930000000</v>
+        <v>108949000000</v>
       </c>
       <c r="E14" s="20" t="n">
-        <v>66288000000</v>
+        <v>119437000000</v>
       </c>
       <c r="F14" s="20" t="n">
-        <v>108949000000</v>
+        <v>114301000000</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>119437000000</v>
+        <v>123216000000</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>114301000000</v>
+        <v>133050000000</v>
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
@@ -1574,13 +1574,13 @@
         </is>
       </c>
       <c r="D16" s="10" t="n">
-        <v>3576000000</v>
+        <v>2645000000</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>2873000000</v>
+        <v>2931000000</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>2645000000</v>
+        <v>3933000000</v>
       </c>
       <c r="G16" s="19" t="inlineStr">
         <is>
@@ -1605,19 +1605,19 @@
         </is>
       </c>
       <c r="D17" s="10" t="n">
-        <v>65737000000</v>
+        <v>109207000000</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>67091000000</v>
+        <v>119103000000</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>109207000000</v>
+        <v>113736000000</v>
       </c>
       <c r="G17" s="10" t="n">
-        <v>119103000000</v>
+        <v>123485000000</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>113736000000</v>
+        <v>132729000000</v>
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
@@ -1632,19 +1632,19 @@
         </is>
       </c>
       <c r="D18" s="10" t="n">
-        <v>10481000000</v>
+        <v>14527000000</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>9680000000</v>
+        <v>19300000000</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>14527000000</v>
+        <v>16741000000</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>19300000000</v>
+        <v>29749000000</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>16741000000</v>
+        <v>20719000000</v>
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
@@ -1659,19 +1659,19 @@
         </is>
       </c>
       <c r="D19" s="20" t="n">
-        <v>55256000000</v>
+        <v>94680000000</v>
       </c>
       <c r="E19" s="20" t="n">
-        <v>57411000000</v>
+        <v>99803000000</v>
       </c>
       <c r="F19" s="20" t="n">
-        <v>94680000000</v>
+        <v>96995000000</v>
       </c>
       <c r="G19" s="20" t="n">
-        <v>99803000000</v>
+        <v>93736000000</v>
       </c>
       <c r="H19" s="20" t="n">
-        <v>96995000000</v>
+        <v>112010000000</v>
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
@@ -1805,19 +1805,19 @@
         </is>
       </c>
       <c r="D7" s="10" t="n">
-        <v>38016000000</v>
+        <v>34940000000</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>34940000000</v>
+        <v>23646000000</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>23646000000</v>
+        <v>29965000000</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>29965000000</v>
+        <v>29943000000</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>29943000000</v>
+        <v>35934000000</v>
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
@@ -1864,19 +1864,19 @@
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>16120000000</v>
+        <v>26278000000</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>26278000000</v>
+        <v>28184000000</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>28184000000</v>
+        <v>29508000000</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>29508000000</v>
+        <v>33410000000</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>33410000000</v>
+        <v>39777000000</v>
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
@@ -1891,19 +1891,19 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>4061000000</v>
+        <v>6580000000</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>6580000000</v>
+        <v>4946000000</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>4946000000</v>
+        <v>6331000000</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>6331000000</v>
+        <v>7286000000</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>7286000000</v>
+        <v>5718000000</v>
       </c>
       <c r="J10" s="11" t="inlineStr">
         <is>
@@ -1918,19 +1918,19 @@
         </is>
       </c>
       <c r="D11" s="20" t="n">
-        <v>143713000000</v>
+        <v>134836000000</v>
       </c>
       <c r="E11" s="20" t="n">
-        <v>134836000000</v>
+        <v>135405000000</v>
       </c>
       <c r="F11" s="20" t="n">
-        <v>135405000000</v>
+        <v>143566000000</v>
       </c>
       <c r="G11" s="20" t="n">
-        <v>143566000000</v>
+        <v>152987000000</v>
       </c>
       <c r="H11" s="20" t="n">
-        <v>152987000000</v>
+        <v>147957000000</v>
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
@@ -1945,19 +1945,19 @@
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>36766000000</v>
+        <v>39440000000</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>39440000000</v>
+        <v>42117000000</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>42117000000</v>
+        <v>43715000000</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>43715000000</v>
+        <v>45680000000</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>45680000000</v>
+        <v>49834000000</v>
       </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
@@ -2004,19 +2004,19 @@
         </is>
       </c>
       <c r="D14" s="20" t="n">
-        <v>323888000000</v>
+        <v>351002000000</v>
       </c>
       <c r="E14" s="20" t="n">
-        <v>351002000000</v>
+        <v>352755000000</v>
       </c>
       <c r="F14" s="20" t="n">
-        <v>352755000000</v>
+        <v>352583000000</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>352583000000</v>
+        <v>364980000000</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>364980000000</v>
+        <v>359241000000</v>
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
@@ -2031,19 +2031,19 @@
         </is>
       </c>
       <c r="D15" s="10" t="n">
-        <v>42296000000</v>
+        <v>54763000000</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>54763000000</v>
+        <v>64115000000</v>
       </c>
       <c r="F15" s="10" t="n">
-        <v>64115000000</v>
+        <v>62611000000</v>
       </c>
       <c r="G15" s="10" t="n">
-        <v>62611000000</v>
+        <v>68960000000</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>68960000000</v>
+        <v>69860000000</v>
       </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
@@ -2058,19 +2058,19 @@
         </is>
       </c>
       <c r="D16" s="20" t="n">
-        <v>105392000000</v>
+        <v>125481000000</v>
       </c>
       <c r="E16" s="20" t="n">
-        <v>125481000000</v>
+        <v>153982000000</v>
       </c>
       <c r="F16" s="20" t="n">
-        <v>153982000000</v>
+        <v>145308000000</v>
       </c>
       <c r="G16" s="20" t="n">
-        <v>145308000000</v>
+        <v>176392000000</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>176392000000</v>
+        <v>165631000000</v>
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
@@ -2085,19 +2085,19 @@
         </is>
       </c>
       <c r="D17" s="10" t="n">
-        <v>8773000000</v>
+        <v>9613000000</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>9613000000</v>
+        <v>11128000000</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>11128000000</v>
+        <v>9822000000</v>
       </c>
       <c r="G17" s="10" t="n">
-        <v>9822000000</v>
+        <v>10912000000</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>10912000000</v>
+        <v>12350000000</v>
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
@@ -2112,19 +2112,19 @@
         </is>
       </c>
       <c r="D18" s="10" t="n">
-        <v>98667000000</v>
+        <v>109106000000</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>109106000000</v>
+        <v>98959000000</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>98959000000</v>
+        <v>95281000000</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>95281000000</v>
+        <v>85750000000</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>85750000000</v>
+        <v>78328000000</v>
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
@@ -2139,19 +2139,19 @@
         </is>
       </c>
       <c r="D19" s="20" t="n">
-        <v>258549000000</v>
+        <v>287912000000</v>
       </c>
       <c r="E19" s="20" t="n">
-        <v>287912000000</v>
+        <v>302083000000</v>
       </c>
       <c r="F19" s="20" t="n">
-        <v>302083000000</v>
+        <v>290437000000</v>
       </c>
       <c r="G19" s="20" t="n">
-        <v>290437000000</v>
+        <v>308030000000</v>
       </c>
       <c r="H19" s="20" t="n">
-        <v>308030000000</v>
+        <v>285508000000</v>
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
@@ -2166,19 +2166,19 @@
         </is>
       </c>
       <c r="D20" s="20" t="n">
-        <v>107147000000</v>
+        <v>63090000000</v>
       </c>
       <c r="E20" s="20" t="n">
-        <v>90488000000</v>
+        <v>50672000000</v>
       </c>
       <c r="F20" s="20" t="n">
-        <v>65339000000</v>
+        <v>62146000000</v>
       </c>
       <c r="G20" s="20" t="n">
-        <v>63090000000</v>
+        <v>56950000000</v>
       </c>
       <c r="H20" s="20" t="n">
-        <v>50672000000</v>
+        <v>73733000000</v>
       </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
@@ -2193,19 +2193,19 @@
         </is>
       </c>
       <c r="D22" s="20" t="n">
-        <v>323888000000</v>
+        <v>351002000000</v>
       </c>
       <c r="E22" s="20" t="n">
-        <v>351002000000</v>
+        <v>352755000000</v>
       </c>
       <c r="F22" s="20" t="n">
-        <v>352755000000</v>
+        <v>352583000000</v>
       </c>
       <c r="G22" s="20" t="n">
-        <v>352583000000</v>
+        <v>364980000000</v>
       </c>
       <c r="H22" s="20" t="n">
-        <v>364980000000</v>
+        <v>359241000000</v>
       </c>
       <c r="J22" s="11" t="inlineStr">
         <is>
@@ -2351,19 +2351,19 @@
         </is>
       </c>
       <c r="D7" s="20" t="n">
-        <v>69391000000</v>
+        <v>104038000000</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>80674000000</v>
+        <v>122151000000</v>
       </c>
       <c r="F7" s="20" t="n">
-        <v>104038000000</v>
+        <v>110543000000</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>122151000000</v>
+        <v>118254000000</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>110543000000</v>
+        <v>111482000000</v>
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
@@ -2378,19 +2378,19 @@
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>10495000000</v>
+        <v>11085000000</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>7309000000</v>
+        <v>10708000000</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>11085000000</v>
+        <v>10959000000</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>10708000000</v>
+        <v>9447000000</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>10959000000</v>
+        <v>12715000000</v>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
@@ -2405,19 +2405,19 @@
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>45896000000</v>
+        <v>-14545000000</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>-4289000000</v>
+        <v>-22354000000</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>-14545000000</v>
+        <v>3705000000</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>-22354000000</v>
+        <v>2935000000</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>3705000000</v>
+        <v>15195000000</v>
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
@@ -2432,19 +2432,19 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>-90976000000</v>
+        <v>-93353000000</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>-86820000000</v>
+        <v>-110749000000</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>-93353000000</v>
+        <v>-108488000000</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>-110749000000</v>
+        <v>-121983000000</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-108488000000</v>
+        <v>-120686000000</v>
       </c>
       <c r="J10" s="11" t="inlineStr">
         <is>
@@ -2459,19 +2459,19 @@
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>66897000000</v>
+        <v>85971000000</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>72358000000</v>
+        <v>89402000000</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>85971000000</v>
+        <v>77550000000</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>89402000000</v>
+        <v>94949000000</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>77550000000</v>
+        <v>90711000000</v>
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:RevenueFromContractWithCustomerExcludingAssessedTax · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:RevenueFromContractWithCustomerExcludingAssessedTax · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E8" s="25" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:RevenueFromContractWithCustomerExcludingAssessedTax · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:RevenueFromContractWithCustomerExcludingAssessedTax · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E9" s="25" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:RevenueFromContractWithCustomerExcludingAssessedTax · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:RevenueFromContractWithCustomerExcludingAssessedTax · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E10" s="25" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="D11" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:RevenueFromContractWithCustomerExcludingAssessedTax · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:RevenueFromContractWithCustomerExcludingAssessedTax · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E11" s="25" t="inlineStr">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:RevenueFromContractWithCustomerExcludingAssessedTax · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:RevenueFromContractWithCustomerExcludingAssessedTax · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E12" s="25" t="inlineStr">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="D13" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:GrossProfit · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:GrossProfit · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E13" s="25" t="inlineStr">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:GrossProfit · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:GrossProfit · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E14" s="25" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="D15" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:GrossProfit · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:GrossProfit · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E15" s="25" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="D16" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:GrossProfit · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:GrossProfit · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E16" s="25" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="D17" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:GrossProfit · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:GrossProfit · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E17" s="25" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="D18" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:OperatingIncomeLoss · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:OperatingIncomeLoss · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E18" s="25" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="D19" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:OperatingIncomeLoss · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:OperatingIncomeLoss · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E19" s="25" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="D20" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:OperatingIncomeLoss · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:OperatingIncomeLoss · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E20" s="25" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="D21" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:OperatingIncomeLoss · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:OperatingIncomeLoss · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E21" s="25" t="inlineStr">
@@ -3171,7 +3171,7 @@
       </c>
       <c r="D22" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:OperatingIncomeLoss · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:OperatingIncomeLoss · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E22" s="25" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="D23" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetIncomeLoss · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:NetIncomeLoss · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E23" s="25" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="D24" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetIncomeLoss · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:NetIncomeLoss · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E24" s="25" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="D25" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetIncomeLoss · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:NetIncomeLoss · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E25" s="25" t="inlineStr">
@@ -3271,7 +3271,7 @@
       </c>
       <c r="D26" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetIncomeLoss · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:NetIncomeLoss · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E26" s="25" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="D27" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetIncomeLoss · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:NetIncomeLoss · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E27" s="25" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="D28" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:EarningsPerShareDiluted · period ending 2019-09-28 · USD/shares · filed 2021-10-29</t>
+          <t>us-gaap:EarningsPerShareDiluted · period ending 2021-09-25 · USD/shares · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E28" s="25" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="D29" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:EarningsPerShareDiluted · period ending 2020-09-26 · USD/shares · filed 2022-10-28</t>
+          <t>us-gaap:EarningsPerShareDiluted · period ending 2022-09-24 · USD/shares · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E29" s="25" t="inlineStr">
@@ -3371,7 +3371,7 @@
       </c>
       <c r="D30" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:EarningsPerShareDiluted · period ending 2021-09-25 · USD/shares · filed 2023-11-03</t>
+          <t>us-gaap:EarningsPerShareDiluted · period ending 2023-09-30 · USD/shares · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E30" s="25" t="inlineStr">
@@ -3396,7 +3396,7 @@
       </c>
       <c r="D31" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:EarningsPerShareDiluted · period ending 2022-09-24 · USD/shares · filed 2024-11-01</t>
+          <t>us-gaap:EarningsPerShareDiluted · period ending 2024-09-28 · USD/shares · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E31" s="25" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="D32" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:EarningsPerShareDiluted · period ending 2023-09-30 · USD/shares · filed 2025-10-31</t>
+          <t>us-gaap:EarningsPerShareDiluted · period ending 2025-09-27 · USD/shares · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E32" s="25" t="inlineStr">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="D33" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:WeightedAverageNumberOfDilutedSharesOutstanding · period ending 2019-09-28 · shares · filed 2021-10-29</t>
+          <t>us-gaap:WeightedAverageNumberOfDilutedSharesOutstanding · period ending 2021-09-25 · shares · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E33" s="25" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="D34" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:WeightedAverageNumberOfDilutedSharesOutstanding · period ending 2020-09-26 · shares · filed 2022-10-28</t>
+          <t>us-gaap:WeightedAverageNumberOfDilutedSharesOutstanding · period ending 2022-09-24 · shares · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E34" s="25" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="D35" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:WeightedAverageNumberOfDilutedSharesOutstanding · period ending 2021-09-25 · shares · filed 2023-11-03</t>
+          <t>us-gaap:WeightedAverageNumberOfDilutedSharesOutstanding · period ending 2023-09-30 · shares · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E35" s="25" t="inlineStr">
@@ -3521,7 +3521,7 @@
       </c>
       <c r="D36" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:WeightedAverageNumberOfDilutedSharesOutstanding · period ending 2022-09-24 · shares · filed 2024-11-01</t>
+          <t>us-gaap:WeightedAverageNumberOfDilutedSharesOutstanding · period ending 2024-09-28 · shares · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E36" s="25" t="inlineStr">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="D37" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:WeightedAverageNumberOfDilutedSharesOutstanding · period ending 2023-09-30 · shares · filed 2025-10-31</t>
+          <t>us-gaap:WeightedAverageNumberOfDilutedSharesOutstanding · period ending 2025-09-27 · shares · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E37" s="25" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="D38" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInOperatingActivities · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:NetCashProvidedByUsedInOperatingActivities · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E38" s="25" t="inlineStr">
@@ -3596,7 +3596,7 @@
       </c>
       <c r="D39" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInOperatingActivities · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:NetCashProvidedByUsedInOperatingActivities · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E39" s="25" t="inlineStr">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="D40" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInOperatingActivities · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:NetCashProvidedByUsedInOperatingActivities · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E40" s="25" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="D41" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInOperatingActivities · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:NetCashProvidedByUsedInOperatingActivities · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E41" s="25" t="inlineStr">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="D42" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInOperatingActivities · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:NetCashProvidedByUsedInOperatingActivities · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E42" s="25" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="D43" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E43" s="25" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="D44" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E44" s="25" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D45" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E45" s="25" t="inlineStr">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="D46" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E46" s="25" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="D47" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E47" s="25" t="inlineStr">
@@ -3821,7 +3821,7 @@
       </c>
       <c r="D48" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:CashAndCashEquivalentsAtCarryingValue · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:CashAndCashEquivalentsAtCarryingValue · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E48" s="25" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="D49" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:CashAndCashEquivalentsAtCarryingValue · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:CashAndCashEquivalentsAtCarryingValue · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E49" s="25" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="D50" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:CashAndCashEquivalentsAtCarryingValue · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:CashAndCashEquivalentsAtCarryingValue · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E50" s="25" t="inlineStr">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="D51" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:CashAndCashEquivalentsAtCarryingValue · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:CashAndCashEquivalentsAtCarryingValue · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E51" s="25" t="inlineStr">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="D52" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:CashAndCashEquivalentsAtCarryingValue · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:CashAndCashEquivalentsAtCarryingValue · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E52" s="25" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="D53" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LongTermDebtNoncurrent · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:LongTermDebtNoncurrent · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E53" s="25" t="inlineStr">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="D54" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LongTermDebtNoncurrent · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:LongTermDebtNoncurrent · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E54" s="25" t="inlineStr">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="D55" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LongTermDebtNoncurrent · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:LongTermDebtNoncurrent · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E55" s="25" t="inlineStr">
@@ -4021,7 +4021,7 @@
       </c>
       <c r="D56" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LongTermDebtNoncurrent · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:LongTermDebtNoncurrent · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E56" s="25" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="D57" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LongTermDebtNoncurrent · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:LongTermDebtNoncurrent · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E57" s="25" t="inlineStr">
@@ -4071,7 +4071,7 @@
       </c>
       <c r="D58" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LongTermDebtCurrent · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:LongTermDebtCurrent · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E58" s="25" t="inlineStr">
@@ -4096,7 +4096,7 @@
       </c>
       <c r="D59" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LongTermDebtCurrent · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:LongTermDebtCurrent · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E59" s="25" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="D60" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LongTermDebtCurrent · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:LongTermDebtCurrent · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E60" s="25" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="D61" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LongTermDebtCurrent · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:LongTermDebtCurrent · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E61" s="25" t="inlineStr">
@@ -4171,7 +4171,7 @@
       </c>
       <c r="D62" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LongTermDebtCurrent · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:LongTermDebtCurrent · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E62" s="25" t="inlineStr">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="D63" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:StockholdersEquity · period ending 2018-09-29 · USD · filed 2021-10-29</t>
+          <t>us-gaap:StockholdersEquity · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E63" s="25" t="inlineStr">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="D64" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:StockholdersEquity · period ending 2019-09-28 · USD · filed 2022-10-28</t>
+          <t>us-gaap:StockholdersEquity · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E64" s="25" t="inlineStr">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="D65" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:StockholdersEquity · period ending 2020-09-26 · USD · filed 2023-11-03</t>
+          <t>us-gaap:StockholdersEquity · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E65" s="25" t="inlineStr">
@@ -4271,7 +4271,7 @@
       </c>
       <c r="D66" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:StockholdersEquity · period ending 2021-09-25 · USD · filed 2024-11-01</t>
+          <t>us-gaap:StockholdersEquity · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E66" s="25" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="D67" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:StockholdersEquity · period ending 2022-09-24 · USD · filed 2025-10-31</t>
+          <t>us-gaap:StockholdersEquity · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E67" s="25" t="inlineStr">
@@ -4321,7 +4321,7 @@
       </c>
       <c r="D68" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:CostOfGoodsAndServicesSold · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:CostOfGoodsAndServicesSold · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E68" s="25" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="D69" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:CostOfGoodsAndServicesSold · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:CostOfGoodsAndServicesSold · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E69" s="25" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="D70" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:CostOfGoodsAndServicesSold · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:CostOfGoodsAndServicesSold · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E70" s="25" t="inlineStr">
@@ -4396,7 +4396,7 @@
       </c>
       <c r="D71" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:CostOfGoodsAndServicesSold · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:CostOfGoodsAndServicesSold · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E71" s="25" t="inlineStr">
@@ -4421,7 +4421,7 @@
       </c>
       <c r="D72" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:CostOfGoodsAndServicesSold · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:CostOfGoodsAndServicesSold · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E72" s="25" t="inlineStr">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="D73" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:ResearchAndDevelopmentExpense · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:ResearchAndDevelopmentExpense · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E73" s="25" t="inlineStr">
@@ -4471,7 +4471,7 @@
       </c>
       <c r="D74" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:ResearchAndDevelopmentExpense · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:ResearchAndDevelopmentExpense · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E74" s="25" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="D75" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:ResearchAndDevelopmentExpense · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:ResearchAndDevelopmentExpense · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E75" s="25" t="inlineStr">
@@ -4521,7 +4521,7 @@
       </c>
       <c r="D76" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:ResearchAndDevelopmentExpense · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:ResearchAndDevelopmentExpense · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E76" s="25" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="D77" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:ResearchAndDevelopmentExpense · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:ResearchAndDevelopmentExpense · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E77" s="25" t="inlineStr">
@@ -4571,7 +4571,7 @@
       </c>
       <c r="D78" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:SellingGeneralAndAdministrativeExpense · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:SellingGeneralAndAdministrativeExpense · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E78" s="25" t="inlineStr">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="D79" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:SellingGeneralAndAdministrativeExpense · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:SellingGeneralAndAdministrativeExpense · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E79" s="25" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="D80" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:SellingGeneralAndAdministrativeExpense · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:SellingGeneralAndAdministrativeExpense · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E80" s="25" t="inlineStr">
@@ -4646,7 +4646,7 @@
       </c>
       <c r="D81" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:SellingGeneralAndAdministrativeExpense · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:SellingGeneralAndAdministrativeExpense · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E81" s="25" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="D82" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:SellingGeneralAndAdministrativeExpense · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:SellingGeneralAndAdministrativeExpense · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E82" s="25" t="inlineStr">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="D83" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:InterestExpense · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:InterestExpense · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E83" s="25" t="inlineStr">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="D84" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:InterestExpense · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:InterestExpense · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E84" s="25" t="inlineStr">
@@ -4746,7 +4746,7 @@
       </c>
       <c r="D85" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:InterestExpense · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:InterestExpense · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E85" s="25" t="inlineStr">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="D86" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E86" s="25" t="inlineStr">
@@ -4796,7 +4796,7 @@
       </c>
       <c r="D87" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E87" s="25" t="inlineStr">
@@ -4821,7 +4821,7 @@
       </c>
       <c r="D88" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E88" s="25" t="inlineStr">
@@ -4846,7 +4846,7 @@
       </c>
       <c r="D89" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E89" s="25" t="inlineStr">
@@ -4871,7 +4871,7 @@
       </c>
       <c r="D90" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E90" s="25" t="inlineStr">
@@ -4896,7 +4896,7 @@
       </c>
       <c r="D91" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:IncomeTaxExpenseBenefit · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:IncomeTaxExpenseBenefit · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E91" s="25" t="inlineStr">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="D92" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:IncomeTaxExpenseBenefit · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:IncomeTaxExpenseBenefit · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E92" s="25" t="inlineStr">
@@ -4946,7 +4946,7 @@
       </c>
       <c r="D93" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:IncomeTaxExpenseBenefit · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:IncomeTaxExpenseBenefit · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E93" s="25" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="D94" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:IncomeTaxExpenseBenefit · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:IncomeTaxExpenseBenefit · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E94" s="25" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="D95" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:IncomeTaxExpenseBenefit · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:IncomeTaxExpenseBenefit · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E95" s="25" t="inlineStr">
@@ -5021,7 +5021,7 @@
       </c>
       <c r="D96" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AccountsReceivableNetCurrent · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:AccountsReceivableNetCurrent · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E96" s="25" t="inlineStr">
@@ -5046,7 +5046,7 @@
       </c>
       <c r="D97" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AccountsReceivableNetCurrent · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:AccountsReceivableNetCurrent · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E97" s="25" t="inlineStr">
@@ -5071,7 +5071,7 @@
       </c>
       <c r="D98" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AccountsReceivableNetCurrent · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:AccountsReceivableNetCurrent · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E98" s="25" t="inlineStr">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="D99" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AccountsReceivableNetCurrent · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:AccountsReceivableNetCurrent · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E99" s="25" t="inlineStr">
@@ -5121,7 +5121,7 @@
       </c>
       <c r="D100" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AccountsReceivableNetCurrent · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:AccountsReceivableNetCurrent · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E100" s="25" t="inlineStr">
@@ -5146,7 +5146,7 @@
       </c>
       <c r="D101" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:InventoryNet · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:InventoryNet · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E101" s="25" t="inlineStr">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="D102" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:InventoryNet · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:InventoryNet · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E102" s="25" t="inlineStr">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="D103" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:InventoryNet · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:InventoryNet · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E103" s="25" t="inlineStr">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="D104" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:InventoryNet · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:InventoryNet · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E104" s="25" t="inlineStr">
@@ -5246,7 +5246,7 @@
       </c>
       <c r="D105" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:InventoryNet · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:InventoryNet · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E105" s="25" t="inlineStr">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="D106" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AssetsCurrent · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:AssetsCurrent · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E106" s="25" t="inlineStr">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="D107" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AssetsCurrent · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:AssetsCurrent · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E107" s="25" t="inlineStr">
@@ -5321,7 +5321,7 @@
       </c>
       <c r="D108" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AssetsCurrent · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:AssetsCurrent · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E108" s="25" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="D109" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AssetsCurrent · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:AssetsCurrent · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E109" s="25" t="inlineStr">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="D110" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AssetsCurrent · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:AssetsCurrent · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E110" s="25" t="inlineStr">
@@ -5396,7 +5396,7 @@
       </c>
       <c r="D111" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PropertyPlantAndEquipmentNet · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:PropertyPlantAndEquipmentNet · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E111" s="25" t="inlineStr">
@@ -5421,7 +5421,7 @@
       </c>
       <c r="D112" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PropertyPlantAndEquipmentNet · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:PropertyPlantAndEquipmentNet · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E112" s="25" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="D113" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PropertyPlantAndEquipmentNet · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:PropertyPlantAndEquipmentNet · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E113" s="25" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="D114" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PropertyPlantAndEquipmentNet · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:PropertyPlantAndEquipmentNet · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E114" s="25" t="inlineStr">
@@ -5496,7 +5496,7 @@
       </c>
       <c r="D115" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PropertyPlantAndEquipmentNet · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:PropertyPlantAndEquipmentNet · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E115" s="25" t="inlineStr">
@@ -5521,7 +5521,7 @@
       </c>
       <c r="D116" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:Assets · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:Assets · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E116" s="25" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="D117" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:Assets · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:Assets · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E117" s="25" t="inlineStr">
@@ -5571,7 +5571,7 @@
       </c>
       <c r="D118" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:Assets · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:Assets · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E118" s="25" t="inlineStr">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="D119" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:Assets · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:Assets · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E119" s="25" t="inlineStr">
@@ -5621,7 +5621,7 @@
       </c>
       <c r="D120" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:Assets · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:Assets · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E120" s="25" t="inlineStr">
@@ -5646,7 +5646,7 @@
       </c>
       <c r="D121" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AccountsPayableCurrent · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:AccountsPayableCurrent · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E121" s="25" t="inlineStr">
@@ -5671,7 +5671,7 @@
       </c>
       <c r="D122" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AccountsPayableCurrent · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:AccountsPayableCurrent · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E122" s="25" t="inlineStr">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="D123" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AccountsPayableCurrent · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:AccountsPayableCurrent · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E123" s="25" t="inlineStr">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="D124" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AccountsPayableCurrent · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:AccountsPayableCurrent · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E124" s="25" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="D125" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:AccountsPayableCurrent · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:AccountsPayableCurrent · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E125" s="25" t="inlineStr">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="D126" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LiabilitiesCurrent · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:LiabilitiesCurrent · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E126" s="25" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="D127" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LiabilitiesCurrent · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:LiabilitiesCurrent · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E127" s="25" t="inlineStr">
@@ -5821,7 +5821,7 @@
       </c>
       <c r="D128" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LiabilitiesCurrent · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:LiabilitiesCurrent · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E128" s="25" t="inlineStr">
@@ -5846,7 +5846,7 @@
       </c>
       <c r="D129" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LiabilitiesCurrent · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:LiabilitiesCurrent · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E129" s="25" t="inlineStr">
@@ -5871,7 +5871,7 @@
       </c>
       <c r="D130" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LiabilitiesCurrent · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:LiabilitiesCurrent · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E130" s="25" t="inlineStr">
@@ -5896,7 +5896,7 @@
       </c>
       <c r="D131" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:Liabilities · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:Liabilities · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E131" s="25" t="inlineStr">
@@ -5921,7 +5921,7 @@
       </c>
       <c r="D132" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:Liabilities · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:Liabilities · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E132" s="25" t="inlineStr">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="D133" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:Liabilities · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:Liabilities · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E133" s="25" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="D134" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:Liabilities · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:Liabilities · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E134" s="25" t="inlineStr">
@@ -5996,7 +5996,7 @@
       </c>
       <c r="D135" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:Liabilities · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:Liabilities · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E135" s="25" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="D136" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LiabilitiesAndStockholdersEquity · period ending 2020-09-26 · USD · filed 2021-10-29</t>
+          <t>us-gaap:LiabilitiesAndStockholdersEquity · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E136" s="25" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="D137" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LiabilitiesAndStockholdersEquity · period ending 2021-09-25 · USD · filed 2022-10-28</t>
+          <t>us-gaap:LiabilitiesAndStockholdersEquity · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E137" s="25" t="inlineStr">
@@ -6071,7 +6071,7 @@
       </c>
       <c r="D138" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LiabilitiesAndStockholdersEquity · period ending 2022-09-24 · USD · filed 2023-11-03</t>
+          <t>us-gaap:LiabilitiesAndStockholdersEquity · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E138" s="25" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="D139" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LiabilitiesAndStockholdersEquity · period ending 2023-09-30 · USD · filed 2024-11-01</t>
+          <t>us-gaap:LiabilitiesAndStockholdersEquity · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E139" s="25" t="inlineStr">
@@ -6121,7 +6121,7 @@
       </c>
       <c r="D140" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:LiabilitiesAndStockholdersEquity · period ending 2024-09-28 · USD · filed 2025-10-31</t>
+          <t>us-gaap:LiabilitiesAndStockholdersEquity · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E140" s="25" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="D141" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInInvestingActivities · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:NetCashProvidedByUsedInInvestingActivities · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E141" s="25" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="D142" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInInvestingActivities · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:NetCashProvidedByUsedInInvestingActivities · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E142" s="25" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="D143" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInInvestingActivities · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:NetCashProvidedByUsedInInvestingActivities · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E143" s="25" t="inlineStr">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="D144" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInInvestingActivities · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:NetCashProvidedByUsedInInvestingActivities · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E144" s="25" t="inlineStr">
@@ -6246,7 +6246,7 @@
       </c>
       <c r="D145" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInInvestingActivities · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:NetCashProvidedByUsedInInvestingActivities · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E145" s="25" t="inlineStr">
@@ -6271,7 +6271,7 @@
       </c>
       <c r="D146" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInFinancingActivities · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:NetCashProvidedByUsedInFinancingActivities · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E146" s="25" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="D147" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInFinancingActivities · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:NetCashProvidedByUsedInFinancingActivities · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E147" s="25" t="inlineStr">
@@ -6321,7 +6321,7 @@
       </c>
       <c r="D148" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInFinancingActivities · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:NetCashProvidedByUsedInFinancingActivities · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E148" s="25" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="D149" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInFinancingActivities · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:NetCashProvidedByUsedInFinancingActivities · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E149" s="25" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="D150" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:NetCashProvidedByUsedInFinancingActivities · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:NetCashProvidedByUsedInFinancingActivities · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E150" s="25" t="inlineStr">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="D151" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PaymentsForRepurchaseOfCommonStock · period ending 2019-09-28 · USD · filed 2021-10-29</t>
+          <t>us-gaap:PaymentsForRepurchaseOfCommonStock · period ending 2021-09-25 · USD · filed 2021-10-29</t>
         </is>
       </c>
       <c r="E151" s="25" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="D152" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PaymentsForRepurchaseOfCommonStock · period ending 2020-09-26 · USD · filed 2022-10-28</t>
+          <t>us-gaap:PaymentsForRepurchaseOfCommonStock · period ending 2022-09-24 · USD · filed 2022-10-28</t>
         </is>
       </c>
       <c r="E152" s="25" t="inlineStr">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="D153" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PaymentsForRepurchaseOfCommonStock · period ending 2021-09-25 · USD · filed 2023-11-03</t>
+          <t>us-gaap:PaymentsForRepurchaseOfCommonStock · period ending 2023-09-30 · USD · filed 2023-11-03</t>
         </is>
       </c>
       <c r="E153" s="25" t="inlineStr">
@@ -6471,7 +6471,7 @@
       </c>
       <c r="D154" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PaymentsForRepurchaseOfCommonStock · period ending 2022-09-24 · USD · filed 2024-11-01</t>
+          <t>us-gaap:PaymentsForRepurchaseOfCommonStock · period ending 2024-09-28 · USD · filed 2024-11-01</t>
         </is>
       </c>
       <c r="E154" s="25" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="D155" s="25" t="inlineStr">
         <is>
-          <t>us-gaap:PaymentsForRepurchaseOfCommonStock · period ending 2023-09-30 · USD · filed 2025-10-31</t>
+          <t>us-gaap:PaymentsForRepurchaseOfCommonStock · period ending 2025-09-27 · USD · filed 2025-10-31</t>
         </is>
       </c>
       <c r="E155" s="25" t="inlineStr">

</xml_diff>